<commit_message>
Refactor button layout in FocusViewWindow and ScanWindow for improved grid management
</commit_message>
<xml_diff>
--- a/Sessions/3rd October session 1.xlsx
+++ b/Sessions/3rd October session 1.xlsx
@@ -935,17 +935,17 @@
           <t>null 9</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>attend</t>
-        </is>
-      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>[00:39:15]</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
+          <t>[01:35:41]</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>[01:35:41] Canceled.</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -988,17 +988,17 @@
           <t>null 10</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>attend</t>
-        </is>
-      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>[00:50:07]</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr"/>
+          <t>[01:35:36]</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>[01:35:36] Canceled.</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -1041,8 +1041,16 @@
           <t>null 11</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>[01:28:28]</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
@@ -1086,8 +1094,16 @@
           <t>null 12</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>[01:31:01]</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
@@ -1132,8 +1148,16 @@
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>[01:31:25]</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>[01:31:25] Canceled.</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -1266,9 +1290,21 @@
           <t>null 16</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>[01:28:39]</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>[01:28:39] Attended (Didn't do Exam &amp; Homework).</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -1303,8 +1339,16 @@
           <t>null 17</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>[01:35:14]</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
@@ -1708,9 +1752,21 @@
           <t>null 26</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>[01:31:11]</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>[01:31:11] Attended (Didn't do Exam &amp; Homework).</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -1745,9 +1801,21 @@
           <t>null 27</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>[01:35:26]</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>[01:35:26] Attended (Didn't do Exam &amp; Homework).</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr">
         <is>
           <t>excel_import</t>

</xml_diff>

<commit_message>
Add Arabic text support and formatting in ScanWindow
</commit_message>
<xml_diff>
--- a/Sessions/3rd October session 1.xlsx
+++ b/Sessions/3rd October session 1.xlsx
@@ -511,19 +511,19 @@
           <t>null 1</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>attend</t>
-        </is>
-      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>[00:32:37]</t>
+          <t>[02:02:25]</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>[00:29:33] Denied Entry: No Exam &amp; Homework.
+[00:32:37] Attended (Didn't do Exam &amp; Homework).
+[00:29:33] Denied Entry: No Exam &amp; Homework.
+[02:02:25] Canceled.
+[00:29:33] Denied Entry: No Exam &amp; Homework.
 [00:32:37] Attended (Didn't do Exam &amp; Homework).
 [00:29:33] Denied Entry: No Exam &amp; Homework.</t>
         </is>
@@ -935,15 +935,20 @@
           <t>null 9</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>[01:35:41]</t>
+          <t>[02:02:34]</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>[01:35:41] Canceled.</t>
+          <t>[01:35:41] Canceled.
+[01:35:41] Canceled.</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1041,17 +1046,17 @@
           <t>null 11</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>attend</t>
-        </is>
-      </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>[01:28:28]</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
+          <t>[02:02:31]</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>[02:02:31] Canceled.</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -1290,19 +1295,17 @@
           <t>null 16</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>attend</t>
-        </is>
-      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>[01:28:39]</t>
+          <t>[01:55:11]</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>[01:28:39] Attended (Didn't do Exam &amp; Homework).</t>
+          <t>[01:28:39] Attended (Didn't do Exam &amp; Homework).
+[01:55:11] Canceled.
+[01:28:39] Attended (Didn't do Exam &amp; Homework).</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1392,8 +1395,16 @@
           <t>null 18</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>[01:41:03]</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
@@ -2681,8 +2692,16 @@
           <t>null 47</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>[01:54:57]</t>
+        </is>
+      </c>
       <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add 's' key press handler to focus scan entry and improve Treeview navigation in ScanWindow
</commit_message>
<xml_diff>
--- a/Sessions/3rd October session 1.xlsx
+++ b/Sessions/3rd October session 1.xlsx
@@ -727,7 +727,7 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>[00:40:08]</t>
+          <t>[02:24:51]</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -746,6 +746,22 @@
 [00:40:05] Completed Exam &amp; Homework at center.
 [00:39:50] Attended (Didn't do Exam &amp; Homework).
 [00:39:58] Canceled.
+[00:39:50] Attended (Didn't do Exam &amp; Homework).
+[02:24:51] Denied Entry: No Exam &amp; Homework.
+[00:39:50] Attended (Didn't do Exam &amp; Homework).
+[00:39:58] Canceled.
+[00:39:50] Attended (Didn't do Exam &amp; Homework).
+[00:40:05] Completed Exam &amp; Homework at center.
+[00:39:50] Attended (Didn't do Exam &amp; Homework).
+[00:39:58] Canceled.
+[00:39:50] Attended (Didn't do Exam &amp; Homework).
+[00:40:08] Canceled.
+[00:39:50] Attended (Didn't do Exam &amp; Homework).
+[00:39:58] Canceled.
+[00:39:50] Attended (Didn't do Exam &amp; Homework).
+[00:40:05] Completed Exam &amp; Homework at center.
+[00:39:50] Attended (Didn't do Exam &amp; Homework).
+[00:39:58] Canceled.
 [00:39:50] Attended (Didn't do Exam &amp; Homework).</t>
         </is>
       </c>

</xml_diff>

<commit_message>
feat: update UI fonts to Roboto for consistency across dialogs and windows
</commit_message>
<xml_diff>
--- a/Sessions/3rd October session 1.xlsx
+++ b/Sessions/3rd October session 1.xlsx
@@ -511,9 +511,21 @@
           <t>null 1</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>03:43:15 AM</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>[03:43:15 AM] Completed Exam &amp; Homework at center.</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -548,8 +560,16 @@
           <t>null 2</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>03:42:18 AM</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
@@ -593,7 +613,11 @@
           <t>null 3</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
@@ -630,7 +654,11 @@
           <t>null 4</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
@@ -675,7 +703,11 @@
           <t>null 5</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
@@ -712,7 +744,11 @@
           <t>null 6</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
@@ -753,7 +789,11 @@
           <t>null 7</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
@@ -798,7 +838,11 @@
           <t>null 8</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
@@ -843,7 +887,11 @@
           <t>null 9</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
@@ -888,7 +936,11 @@
           <t>null 10</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
@@ -933,7 +985,11 @@
           <t>null 11</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
@@ -978,7 +1034,11 @@
           <t>null 12</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
@@ -1023,7 +1083,11 @@
           <t>null 13</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
@@ -1068,7 +1132,11 @@
           <t>null 14</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
@@ -1113,7 +1181,11 @@
           <t>null 15</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
@@ -1158,7 +1230,11 @@
           <t>null 16</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
@@ -1195,7 +1271,11 @@
           <t>null 17</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
@@ -1240,7 +1320,11 @@
           <t>null 18</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
@@ -1285,7 +1369,11 @@
           <t>null 19</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
@@ -1330,7 +1418,11 @@
           <t>null 20</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
@@ -1375,7 +1467,11 @@
           <t>null 21</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
@@ -1420,7 +1516,11 @@
           <t>null 22</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
@@ -1465,7 +1565,11 @@
           <t>null 23</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
@@ -1510,7 +1614,11 @@
           <t>null 24</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
@@ -1555,7 +1663,11 @@
           <t>null 25</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
@@ -1600,7 +1712,11 @@
           <t>null 26</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
@@ -1637,7 +1753,11 @@
           <t>null 27</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
@@ -1674,7 +1794,11 @@
           <t>null 28</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
@@ -1719,7 +1843,11 @@
           <t>null 29</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
@@ -1764,7 +1892,11 @@
           <t>null 30</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
@@ -1809,7 +1941,11 @@
           <t>null 31</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
@@ -1846,7 +1982,11 @@
           <t>null 32</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
@@ -1891,7 +2031,11 @@
           <t>null 33</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
@@ -1936,7 +2080,11 @@
           <t>null 34</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
@@ -1981,7 +2129,11 @@
           <t>null 35</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
@@ -2018,7 +2170,11 @@
           <t>null 36</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
@@ -2055,7 +2211,11 @@
           <t>null 37</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
@@ -2100,7 +2260,11 @@
           <t>null 38</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
@@ -2145,7 +2309,11 @@
           <t>null 39</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
@@ -2190,7 +2358,11 @@
           <t>null 40</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
@@ -2235,7 +2407,11 @@
           <t>null 41</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
@@ -2280,7 +2456,11 @@
           <t>null 42</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
@@ -2325,7 +2505,11 @@
           <t>null 43</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
@@ -2370,7 +2554,11 @@
           <t>null 44</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
@@ -2415,7 +2603,11 @@
           <t>null 45</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
@@ -2460,7 +2652,11 @@
           <t>null 46</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr"/>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr">
@@ -2505,7 +2701,11 @@
           <t>null 47</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr">
@@ -2550,7 +2750,11 @@
           <t>null 48</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr"/>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
@@ -2595,7 +2799,11 @@
           <t>null 49</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr"/>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr">
@@ -2640,7 +2848,11 @@
           <t>null 50</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
@@ -2685,7 +2897,11 @@
           <t>null 51</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr"/>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
@@ -2722,7 +2938,11 @@
           <t>null 52</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr">
@@ -2767,7 +2987,11 @@
           <t>null 53</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
@@ -2808,7 +3032,11 @@
           <t>null 54</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
@@ -2845,7 +3073,11 @@
           <t>null 55</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr">
@@ -2890,7 +3122,11 @@
           <t>null 56</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
@@ -2935,7 +3171,11 @@
           <t>null 57</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr">
@@ -2980,7 +3220,11 @@
           <t>null 58</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr"/>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr">
@@ -3025,7 +3269,11 @@
           <t>null 59</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr">
@@ -3070,7 +3318,11 @@
           <t>null 60</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
@@ -3115,7 +3367,11 @@
           <t>null 61</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr">
@@ -3160,7 +3416,11 @@
           <t>null 62</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr">
@@ -3201,7 +3461,11 @@
           <t>null 63</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr">
@@ -3238,7 +3502,11 @@
           <t>null 64</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr">
@@ -3275,7 +3543,11 @@
           <t>null 65</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr">
@@ -3320,7 +3592,11 @@
           <t>null 66</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
@@ -3365,7 +3641,11 @@
           <t>null 67</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr"/>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr"/>
       <c r="I68" t="inlineStr">
@@ -3410,7 +3690,11 @@
           <t>null 68</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr"/>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr">
@@ -3455,7 +3739,11 @@
           <t>null 69</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr"/>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr"/>
       <c r="I70" t="inlineStr">
@@ -3500,7 +3788,11 @@
           <t>null 70</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr"/>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr"/>
       <c r="I71" t="inlineStr">
@@ -3545,7 +3837,11 @@
           <t>null 71</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr"/>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr"/>
       <c r="I72" t="inlineStr">
@@ -3582,7 +3878,11 @@
           <t>null 72</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr"/>
       <c r="I73" t="inlineStr">
@@ -3627,7 +3927,11 @@
           <t>null 73</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr"/>
       <c r="I74" t="inlineStr">
@@ -3672,7 +3976,11 @@
           <t>null 74</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr">
@@ -3717,7 +4025,11 @@
           <t>null 75</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr"/>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr"/>
       <c r="I76" t="inlineStr">
@@ -3762,7 +4074,11 @@
           <t>null 76</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr"/>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr">
@@ -3803,7 +4119,11 @@
           <t>null 77</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr"/>
       <c r="I78" t="inlineStr">
@@ -3848,7 +4168,11 @@
           <t>null 78</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr"/>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr"/>
       <c r="I79" t="inlineStr">
@@ -3885,7 +4209,11 @@
           <t>null 79</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr"/>
       <c r="I80" t="inlineStr">
@@ -3930,7 +4258,11 @@
           <t>null 80</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr">
@@ -3975,7 +4307,11 @@
           <t>null 81</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr"/>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr"/>
       <c r="I82" t="inlineStr">
@@ -4020,7 +4356,11 @@
           <t>null 82</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr"/>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr"/>
       <c r="I83" t="inlineStr">
@@ -4065,7 +4405,11 @@
           <t>null 83</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr"/>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr"/>
       <c r="I84" t="inlineStr">
@@ -4110,7 +4454,11 @@
           <t>null 84</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr"/>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr"/>
       <c r="I85" t="inlineStr">
@@ -4155,7 +4503,11 @@
           <t>null 85</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr"/>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr"/>
       <c r="I86" t="inlineStr">
@@ -4192,7 +4544,11 @@
           <t>null 86</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr"/>
       <c r="I87" t="inlineStr">
@@ -4229,7 +4585,11 @@
           <t>null 87</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr"/>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr"/>
       <c r="I88" t="inlineStr">
@@ -4274,7 +4634,11 @@
           <t>null 88</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr"/>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr">
@@ -4315,7 +4679,11 @@
           <t>null 89</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr"/>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr"/>
       <c r="I90" t="inlineStr">
@@ -4356,7 +4724,11 @@
           <t>null 90</t>
         </is>
       </c>
-      <c r="F91" t="inlineStr"/>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr"/>
       <c r="I91" t="inlineStr">
@@ -4393,7 +4765,11 @@
           <t>null 91</t>
         </is>
       </c>
-      <c r="F92" t="inlineStr"/>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr"/>
       <c r="I92" t="inlineStr">
@@ -4430,7 +4806,11 @@
           <t>null 92</t>
         </is>
       </c>
-      <c r="F93" t="inlineStr"/>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr">
@@ -4475,7 +4855,11 @@
           <t>null 93</t>
         </is>
       </c>
-      <c r="F94" t="inlineStr"/>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr"/>
       <c r="I94" t="inlineStr">
@@ -4520,7 +4904,11 @@
           <t>null 94</t>
         </is>
       </c>
-      <c r="F95" t="inlineStr"/>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr"/>
       <c r="I95" t="inlineStr">
@@ -4557,7 +4945,11 @@
           <t>null 95</t>
         </is>
       </c>
-      <c r="F96" t="inlineStr"/>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr"/>
       <c r="I96" t="inlineStr"/>
@@ -4590,7 +4982,11 @@
           <t>null 96</t>
         </is>
       </c>
-      <c r="F97" t="inlineStr"/>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr"/>

</xml_diff>